<commit_message>
Refactor: NiceGUI UI, flexible column schema, updated build pipeline
- Rewrites main.py to use NiceGUI native mode instead of tkinter
- Creates ui/app_ui.py with full AppUI class (file pickers, progress queue, result chips)
- Creates ui/styles.py with Apple/macOS-style CSS constants (already existed, confirmed)
- Creates ui/__init__.py (empty module marker)
- Updates requirements.txt to include nicegui[native], pywebview
- Rewrites build.spec to bundle NiceGUI assets via PyInstaller
- Updates GitHub Actions workflow to install NiceGUI deps and use build.spec
- Adds Spital Thurgau AG and TOPAZ-1 entries to master_config.xlsx via create_test_data.py
- Adds test_alt_input.csv and test_alt_expected.csv for alternative column format
- Adds TestFlexibleColumns test class with 5 new tests covering extra/missing columns and ordering
- Updates TestFullPipeline comparison to be robust to output column ordering

https://claude.ai/code/session_01RaXYyRBtZcsJVwhrx7HetF
</commit_message>
<xml_diff>
--- a/claim_cleaner/config_files/master_config.xlsx
+++ b/claim_cleaner/config_files/master_config.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -579,118 +579,130 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Metastatic Breast Cancer, HR+, HER2-, BRCA+ (OlympiAD)  </t>
+          <t>Metastatic distal cholangiocarcinoma (TOPAZ-1)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>OlympiAD</t>
+          <t>TOPAZ-1</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Adjuvant Breast Cancer, triple negative BRCA+ (OlympiA)  </t>
+          <t xml:space="preserve">Metastatic Breast Cancer, HR+, HER2-, BRCA+ (OlympiAD)  </t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>OlympiA</t>
+          <t>OlympiAD</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">ES SCLC 1L plus platinum–etoposide (CASPIAN)  </t>
+          <t xml:space="preserve">Adjuvant Breast Cancer, triple negative BRCA+ (OlympiA)  </t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>CASPIAN</t>
+          <t>OlympiA</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Advanced Ovarian Cancer 1L with Bev after platinum CTx+Bev (PAOLA-1)  </t>
+          <t xml:space="preserve">ES SCLC 1L plus platinum–etoposide (CASPIAN)  </t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>PAOLA-1</t>
+          <t>CASPIAN</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ovarian Cancer, PSR 2L+  </t>
+          <t xml:space="preserve">Advanced Ovarian Cancer 1L with Bev after platinum CTx+Bev (PAOLA-1)  </t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Ovarian Cancer, PSR 2L+</t>
+          <t>PAOLA-1</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Severe Asthma with exacerbations as add on  </t>
+          <t xml:space="preserve">Ovarian Cancer, PSR 2L+  </t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Severe Asthma with exacerbations as add on</t>
+          <t>Ovarian Cancer, PSR 2L+</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Combination with Entresto  </t>
+          <t xml:space="preserve">Severe Asthma with exacerbations as add on  </t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Combination with Entresto</t>
+          <t>Severe Asthma with exacerbations as add on</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Prostate Cancer  </t>
+          <t xml:space="preserve">Combination with Entresto  </t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Prostate Cancer</t>
+          <t>Combination with Entresto</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tezspire-off-Limitatio  </t>
+          <t xml:space="preserve">Prostate Cancer  </t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Tezspire-off-Limitatio</t>
+          <t>Prostate Cancer</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
+          <t xml:space="preserve">Tezspire-off-Limitatio  </t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Tezspire-off-Limitatio</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
           <t xml:space="preserve">NSCLC EGFR+ 1L (Monotherapie) (FLAURA) (SL)  </t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>FLAURA</t>
         </is>
@@ -1023,7 +1035,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1251,6 +1263,18 @@
       <c r="B19" t="inlineStr">
         <is>
           <t>HOCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Spital Thurgau AG</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Spital Thurgau</t>
         </is>
       </c>
     </row>

</xml_diff>